<commit_message>
Strengthen deep learning calculation demos
</commit_message>
<xml_diff>
--- a/02_activation_functions/excel_activation_functions_demo.xlsx
+++ b/02_activation_functions/excel_activation_functions_demo.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,8 +73,16 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F2937"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -101,8 +109,23 @@
         <fgColor rgb="00FFF7CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F4EF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F6F9F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -138,11 +161,25 @@
         <color rgb="00D6B656"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9E2EF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9E2EF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9E2EF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9E2EF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -203,6 +240,27 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -572,7 +630,7 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="88" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -587,7 +645,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>ExcelをUIにして、外部PythonがWorkbookの値を読み、活性化関数とSoftmaxを計算します。</t>
+          <t>Sigmoid、tanh、ReLU、Softmaxの出力と勾配を確認します。SoftmaxとCross Entropyを合わせたときの p - y も表で確認します。</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -619,7 +677,7 @@
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>今回のゴール</t>
+          <t>01_INPUT の input_value、logit、target_class、selected_function、temperature、display_modeを変更してPythonを再実行します。</t>
         </is>
       </c>
       <c r="B5" s="15" t="inlineStr">
@@ -631,7 +689,7 @@
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
         <is>
-          <t>変更する場所</t>
+          <t>display_mode は activation / softmax / softmax_ce_grad / gradient / exam から選びます。</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
@@ -680,16 +738,16 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="4" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="54" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="22" customHeight="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
           <t>第2回 活性化関数: 入力と設定</t>
@@ -704,10 +762,10 @@
       <c r="H1" s="2" t="n"/>
       <c r="I1" s="2" t="n"/>
     </row>
-    <row r="2">
+    <row r="2" ht="34" customHeight="1">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>このシートの表をPythonが xl(...) で読みます。まず display_mode=activation のまま実行してください。</t>
+          <t>このシートの表をPythonが xl(...) で読みます。入力値、logit、正解クラス、表示設定を変えて結果の変化を確認します。</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -719,7 +777,7 @@
       <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
     </row>
-    <row r="3">
+    <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="n"/>
       <c r="B3" s="2" t="n"/>
       <c r="C3" s="2" t="n"/>
@@ -730,22 +788,22 @@
       <c r="H3" s="2" t="n"/>
       <c r="I3" s="2" t="n"/>
     </row>
-    <row r="4">
-      <c r="A4" s="16" t="inlineStr">
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>活性化関数の入力</t>
         </is>
       </c>
       <c r="B4" s="5" t="n"/>
       <c r="C4" s="2" t="n"/>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="D4" s="21" t="inlineStr">
         <is>
           <t>Softmax用logit</t>
         </is>
       </c>
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="2" t="n"/>
-      <c r="G4" s="17" t="inlineStr">
+      <c r="G4" s="21" t="inlineStr">
         <is>
           <t>表示設定</t>
         </is>
@@ -753,7 +811,7 @@
       <c r="H4" s="6" t="n"/>
       <c r="I4" s="6" t="n"/>
     </row>
-    <row r="5">
+    <row r="5" ht="22" customHeight="1">
       <c r="A5" s="2" t="n"/>
       <c r="B5" s="2" t="n"/>
       <c r="C5" s="2" t="n"/>
@@ -764,172 +822,184 @@
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="2" t="n"/>
     </row>
-    <row r="6">
-      <c r="A6" s="14" t="inlineStr">
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>input_id</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>input_value</t>
         </is>
       </c>
       <c r="C6" s="2" t="n"/>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="D6" s="22" t="inlineStr">
         <is>
           <t>class_name</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
+      <c r="E6" s="22" t="inlineStr">
         <is>
           <t>logit</t>
         </is>
       </c>
       <c r="F6" s="2" t="n"/>
-      <c r="G6" s="14" t="inlineStr">
+      <c r="G6" s="22" t="inlineStr">
         <is>
           <t>setting</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr">
+      <c r="H6" s="22" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
+      <c r="I6" s="22" t="inlineStr">
         <is>
           <t>meaning</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="23" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="B7" s="15" t="n">
+      <c r="B7" s="24" t="n">
         <v>-4</v>
       </c>
       <c r="C7" s="2" t="n"/>
-      <c r="D7" s="15" t="inlineStr">
+      <c r="D7" s="23" t="inlineStr">
         <is>
           <t>class_A</t>
         </is>
       </c>
-      <c r="E7" s="15" t="n">
+      <c r="E7" s="24" t="n">
         <v>1.2</v>
       </c>
       <c r="F7" s="2" t="n"/>
-      <c r="G7" s="15" t="inlineStr">
+      <c r="G7" s="25" t="inlineStr">
         <is>
           <t>display_mode</t>
         </is>
       </c>
-      <c r="H7" s="18" t="inlineStr">
+      <c r="H7" s="26" t="inlineStr">
         <is>
           <t>activation</t>
         </is>
       </c>
-      <c r="I7" s="15" t="inlineStr">
-        <is>
-          <t>リストから選択: activation / softmax / gradient / exam</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="I7" s="25" t="inlineStr">
+        <is>
+          <t>リストから選択: activation / softmax / softmax_ce_grad / gradient / exam</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t>v2</t>
         </is>
       </c>
-      <c r="B8" s="15" t="n">
+      <c r="B8" s="24" t="n">
         <v>-2</v>
       </c>
       <c r="C8" s="2" t="n"/>
-      <c r="D8" s="15" t="inlineStr">
+      <c r="D8" s="23" t="inlineStr">
         <is>
           <t>class_B</t>
         </is>
       </c>
-      <c r="E8" s="15" t="n">
+      <c r="E8" s="24" t="n">
         <v>0.4</v>
       </c>
       <c r="F8" s="2" t="n"/>
-      <c r="G8" s="15" t="inlineStr">
+      <c r="G8" s="25" t="inlineStr">
         <is>
           <t>selected_function</t>
         </is>
       </c>
-      <c r="H8" s="18" t="inlineStr">
+      <c r="H8" s="26" t="inlineStr">
         <is>
           <t>relu</t>
         </is>
       </c>
-      <c r="I8" s="15" t="inlineStr">
+      <c r="I8" s="25" t="inlineStr">
         <is>
           <t>リストから選択: sigmoid / tanh / relu</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t>v3</t>
         </is>
       </c>
-      <c r="B9" s="15" t="n">
+      <c r="B9" s="24" t="n">
         <v>-1</v>
       </c>
       <c r="C9" s="2" t="n"/>
-      <c r="D9" s="15" t="inlineStr">
+      <c r="D9" s="23" t="inlineStr">
         <is>
           <t>class_C</t>
         </is>
       </c>
-      <c r="E9" s="15" t="n">
+      <c r="E9" s="24" t="n">
         <v>-0.8</v>
       </c>
       <c r="F9" s="2" t="n"/>
-      <c r="G9" s="15" t="inlineStr">
+      <c r="G9" s="25" t="inlineStr">
         <is>
           <t>temperature</t>
         </is>
       </c>
-      <c r="H9" s="15" t="n">
+      <c r="H9" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="I9" s="15" t="inlineStr">
+      <c r="I9" s="25" t="inlineStr">
         <is>
           <t>Softmaxの尖り方</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="15" t="inlineStr">
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="23" t="inlineStr">
         <is>
           <t>v4</t>
         </is>
       </c>
-      <c r="B10" s="15" t="n">
+      <c r="B10" s="24" t="n">
         <v>0</v>
       </c>
       <c r="C10" s="2" t="n"/>
       <c r="D10" s="2" t="n"/>
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="2" t="n"/>
-      <c r="G10" s="2" t="n"/>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="G10" s="25" t="inlineStr">
+        <is>
+          <t>target_class</t>
+        </is>
+      </c>
+      <c r="H10" s="27" t="inlineStr">
+        <is>
+          <t>class_A</t>
+        </is>
+      </c>
+      <c r="I10" s="25" t="inlineStr">
+        <is>
+          <t>Softmax+CE勾配で使う正解クラス</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="23" t="inlineStr">
         <is>
           <t>v5</t>
         </is>
       </c>
-      <c r="B11" s="15" t="n">
+      <c r="B11" s="24" t="n">
         <v>0.5</v>
       </c>
       <c r="C11" s="2" t="n"/>
@@ -940,13 +1010,13 @@
       <c r="H11" s="2" t="n"/>
       <c r="I11" s="2" t="n"/>
     </row>
-    <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t>v6</t>
         </is>
       </c>
-      <c r="B12" s="15" t="n">
+      <c r="B12" s="24" t="n">
         <v>1</v>
       </c>
       <c r="C12" s="2" t="n"/>
@@ -957,13 +1027,13 @@
       <c r="H12" s="2" t="n"/>
       <c r="I12" s="2" t="n"/>
     </row>
-    <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t>v7</t>
         </is>
       </c>
-      <c r="B13" s="15" t="n">
+      <c r="B13" s="24" t="n">
         <v>2</v>
       </c>
       <c r="C13" s="2" t="n"/>
@@ -974,13 +1044,13 @@
       <c r="H13" s="2" t="n"/>
       <c r="I13" s="2" t="n"/>
     </row>
-    <row r="14">
-      <c r="A14" s="15" t="inlineStr">
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="23" t="inlineStr">
         <is>
           <t>v8</t>
         </is>
       </c>
-      <c r="B14" s="15" t="n">
+      <c r="B14" s="24" t="n">
         <v>4</v>
       </c>
       <c r="C14" s="2" t="n"/>
@@ -991,13 +1061,20 @@
       <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="n"/>
     </row>
+    <row r="15" ht="22" customHeight="1"/>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation sqref="H7" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="リストから選択してください" error="このセルは手入力ではなく、右側のリストから選択します。" promptTitle="選択式の設定" prompt="候補から選ぶと、Pythonの返す表や計算条件が切り替わります。" type="list">
-      <formula1>"activation,softmax,gradient,exam"</formula1>
+  <dataValidations count="4">
+    <dataValidation sqref="H7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"activation,softmax,softmax_ce_grad,gradient,exam"</formula1>
     </dataValidation>
-    <dataValidation sqref="H8" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" errorTitle="リストから選択してください" error="このセルは手入力ではなく、右側のリストから選択します。" promptTitle="選択式の設定" prompt="候補から選ぶと、Pythonの返す表や計算条件が切り替わります。" type="list">
+    <dataValidation sqref="H8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"sigmoid,tanh,relu"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"0.5,1,2"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"class_A,class_B,class_C"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1013,8 +1090,8 @@
   <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
@@ -1022,7 +1099,7 @@
     <row r="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>初期値での確認結果</t>
+          <t>第2回 補強後の確認ポイント</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -1042,12 +1119,12 @@
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>class_name</t>
+          <t>softmax_ce_grad_df</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>logit</t>
+          <t>SoftmaxとCross Entropyを合わせた勾配 p - y を確認する</t>
         </is>
       </c>
       <c r="C3" s="14" t="inlineStr">
@@ -1124,7 +1201,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1138,7 +1215,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>このシートはPython in Excelの実行手順だけを置きます。概念説明はスライドとREADMEで確認します。</t>
+          <t>このシートは実行手順だけを置きます。概念説明はスライドとREADMEで確認します。</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1201,7 +1278,7 @@
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>01_INPUT の display_mode や selected_function を変えて再実行する</t>
+          <t>01_INPUT の display_mode を activation / softmax / softmax_ce_grad / gradient / exam に変えて再実行する</t>
         </is>
       </c>
     </row>

</xml_diff>